<commit_message>
Reviewer 3 robustness runs, script updates, and workspace cleanup
Add outputs from Reviewer 3 full-chain MAF runs (seeds 123/456), updated
evaluation and simulation scripts, revised README, and remove archived
paper/dissertation directories from the repo.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/results/chronological/consolidated/NF_GARCH_Results_chronological.xlsx
+++ b/results/chronological/consolidated/NF_GARCH_Results_chronological.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t xml:space="preserve">Model</t>
   </si>
@@ -54,46 +54,28 @@
     <t xml:space="preserve">std</t>
   </si>
   <si>
+    <t xml:space="preserve">EURUSD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chrono</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GBPUSD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDZAR</t>
+  </si>
+  <si>
     <t xml:space="preserve">NVDA</t>
   </si>
   <si>
-    <t xml:space="preserve">Chrono</t>
-  </si>
-  <si>
     <t xml:space="preserve">MSFT</t>
   </si>
   <si>
-    <t xml:space="preserve">PG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WMT</t>
-  </si>
-  <si>
     <t xml:space="preserve">AMZN</t>
   </si>
   <si>
     <t xml:space="preserve">eGARCH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EURUSD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GBPUSD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GBPCNY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USDZAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GBPZAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EURZAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAT</t>
   </si>
   <si>
     <t xml:space="preserve">gjrGARCH</t>
@@ -498,22 +480,22 @@
         <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>-13207.8962469027</v>
+        <v>-21728.6026698585</v>
       </c>
       <c r="E2" t="n">
-        <v>-13177.9756371092</v>
+        <v>-21698.682060065</v>
       </c>
       <c r="F2" t="n">
-        <v>6608.94812345134</v>
+        <v>10869.3013349292</v>
       </c>
       <c r="G2" t="n">
-        <v>0.00111700386936028</v>
+        <v>0.0000224027333845327</v>
       </c>
       <c r="H2" t="n">
-        <v>0.024321574545893</v>
+        <v>0.00353451751831958</v>
       </c>
       <c r="I2" t="n">
-        <v>1051.6138570919</v>
+        <v>6142.22436264676</v>
       </c>
       <c r="J2" t="n">
         <v>100</v>
@@ -533,22 +515,22 @@
         <v>15</v>
       </c>
       <c r="D3" t="n">
-        <v>-16688.7587376761</v>
+        <v>-22032.0789112467</v>
       </c>
       <c r="E3" t="n">
-        <v>-16658.8381278826</v>
+        <v>-22002.1583014532</v>
       </c>
       <c r="F3" t="n">
-        <v>8349.37936883806</v>
+        <v>11021.0394556234</v>
       </c>
       <c r="G3" t="n">
-        <v>0.000358697849032201</v>
+        <v>0.0000344407971236953</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0133369693265131</v>
+        <v>0.00432584064289235</v>
       </c>
       <c r="I3" t="n">
-        <v>2713.67013051358</v>
+        <v>5308.49589874293</v>
       </c>
       <c r="J3" t="n">
         <v>100</v>
@@ -568,22 +550,22 @@
         <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>-19157.8116926813</v>
+        <v>-18313.964663108</v>
       </c>
       <c r="E4" t="n">
-        <v>-19127.8910828878</v>
+        <v>-18284.0440533145</v>
       </c>
       <c r="F4" t="n">
-        <v>9583.90584634064</v>
+        <v>9161.98233155399</v>
       </c>
       <c r="G4" t="n">
-        <v>0.000173111873391171</v>
+        <v>0.0000991180748912658</v>
       </c>
       <c r="H4" t="n">
-        <v>0.00874978208811587</v>
+        <v>0.00767035118884774</v>
       </c>
       <c r="I4" t="n">
-        <v>3491.92893835333</v>
+        <v>4830.40289359104</v>
       </c>
       <c r="J4" t="n">
         <v>100</v>
@@ -603,22 +585,22 @@
         <v>17</v>
       </c>
       <c r="D5" t="n">
-        <v>-18235.7141496069</v>
+        <v>-13207.8962469027</v>
       </c>
       <c r="E5" t="n">
-        <v>-18205.7935398134</v>
+        <v>-13177.9756371092</v>
       </c>
       <c r="F5" t="n">
-        <v>9122.85707480347</v>
+        <v>6608.94812345134</v>
       </c>
       <c r="G5" t="n">
-        <v>0.000204620345555354</v>
+        <v>0.00111511682117678</v>
       </c>
       <c r="H5" t="n">
-        <v>0.00923064946184809</v>
+        <v>0.0242840606817232</v>
       </c>
       <c r="I5" t="n">
-        <v>4307.42738229818</v>
+        <v>1048.27901233449</v>
       </c>
       <c r="J5" t="n">
         <v>100</v>
@@ -638,22 +620,22 @@
         <v>18</v>
       </c>
       <c r="D6" t="n">
-        <v>-14446.3970235722</v>
+        <v>-16688.7587376761</v>
       </c>
       <c r="E6" t="n">
-        <v>-14416.4764137787</v>
+        <v>-16658.8381278826</v>
       </c>
       <c r="F6" t="n">
-        <v>7228.19851178609</v>
+        <v>8349.37936883806</v>
       </c>
       <c r="G6" t="n">
-        <v>0.000497755201730647</v>
+        <v>0.000358150315451427</v>
       </c>
       <c r="H6" t="n">
-        <v>0.015878292761408</v>
+        <v>0.0133212748572315</v>
       </c>
       <c r="I6" t="n">
-        <v>2923.99885192463</v>
+        <v>2727.83162093552</v>
       </c>
       <c r="J6" t="n">
         <v>100</v>
@@ -664,31 +646,31 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" t="s">
-        <v>20</v>
-      </c>
       <c r="D7" t="n">
-        <v>-21640.2971385716</v>
+        <v>-14446.3970235722</v>
       </c>
       <c r="E7" t="n">
-        <v>-21604.3924068193</v>
+        <v>-14416.4764137787</v>
       </c>
       <c r="F7" t="n">
-        <v>10826.1485692858</v>
+        <v>7228.19851178609</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0000223532175008213</v>
+        <v>0.00049961267719925</v>
       </c>
       <c r="H7" t="n">
-        <v>0.00352284970559203</v>
+        <v>0.0158610810792204</v>
       </c>
       <c r="I7" t="n">
-        <v>6201.41834791827</v>
+        <v>2902.32377923476</v>
       </c>
       <c r="J7" t="n">
         <v>100</v>
@@ -699,31 +681,31 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D8" t="n">
-        <v>-21775.2300244312</v>
+        <v>-21640.2971385716</v>
       </c>
       <c r="E8" t="n">
-        <v>-21739.325292679</v>
+        <v>-21604.3924068193</v>
       </c>
       <c r="F8" t="n">
-        <v>10893.6150122156</v>
+        <v>10826.1485692858</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0000344963526848082</v>
+        <v>0.0000221608514271432</v>
       </c>
       <c r="H8" t="n">
-        <v>0.00433578637453133</v>
+        <v>0.00351249220283315</v>
       </c>
       <c r="I8" t="n">
-        <v>5737.89301323989</v>
+        <v>6189.34866408105</v>
       </c>
       <c r="J8" t="n">
         <v>100</v>
@@ -734,31 +716,31 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D9" t="n">
-        <v>-21710.3566868651</v>
+        <v>-21775.2300244312</v>
       </c>
       <c r="E9" t="n">
-        <v>-21674.4519551129</v>
+        <v>-21739.325292679</v>
       </c>
       <c r="F9" t="n">
-        <v>10861.1783434325</v>
+        <v>10893.6150122156</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0000304993461572959</v>
+        <v>0.0000345894944181152</v>
       </c>
       <c r="H9" t="n">
-        <v>0.00408855784322493</v>
+        <v>0.00434728496418727</v>
       </c>
       <c r="I9" t="n">
-        <v>5887.06846898562</v>
+        <v>5776.93332003491</v>
       </c>
       <c r="J9" t="n">
         <v>100</v>
@@ -769,13 +751,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D10" t="n">
         <v>-18252.5240091211</v>
@@ -787,13 +769,13 @@
         <v>9132.26200456054</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0000997138709326372</v>
+        <v>0.0000985973380235089</v>
       </c>
       <c r="H10" t="n">
-        <v>0.00768966260579867</v>
+        <v>0.00760761934079063</v>
       </c>
       <c r="I10" t="n">
-        <v>5020.223623959</v>
+        <v>5026.77483860042</v>
       </c>
       <c r="J10" t="n">
         <v>100</v>
@@ -804,31 +786,31 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D11" t="n">
-        <v>-18969.8598262053</v>
+        <v>-12886.6841895632</v>
       </c>
       <c r="E11" t="n">
-        <v>-18933.9550944531</v>
+        <v>-12850.779457811</v>
       </c>
       <c r="F11" t="n">
-        <v>9490.92991310267</v>
+        <v>6449.34209478161</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0000812928951129839</v>
+        <v>0.00111967283469879</v>
       </c>
       <c r="H11" t="n">
-        <v>0.00681279691536502</v>
+        <v>0.0243466172036207</v>
       </c>
       <c r="I11" t="n">
-        <v>5145.01998269581</v>
+        <v>2751.62469804481</v>
       </c>
       <c r="J11" t="n">
         <v>100</v>
@@ -839,31 +821,31 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D12" t="n">
-        <v>-19117.2648737316</v>
+        <v>-16459.2335450459</v>
       </c>
       <c r="E12" t="n">
-        <v>-19081.3601419793</v>
+        <v>-16423.3288132937</v>
       </c>
       <c r="F12" t="n">
-        <v>9564.63243686578</v>
+        <v>8235.61677252294</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0000763994832086453</v>
+        <v>0.000358507906132368</v>
       </c>
       <c r="H12" t="n">
-        <v>0.00663780427291206</v>
+        <v>0.0133533408540081</v>
       </c>
       <c r="I12" t="n">
-        <v>5188.01710349232</v>
+        <v>3687.59029229577</v>
       </c>
       <c r="J12" t="n">
         <v>100</v>
@@ -874,31 +856,31 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
         <v>19</v>
       </c>
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" t="s">
-        <v>13</v>
-      </c>
       <c r="D13" t="n">
-        <v>-12886.6841895632</v>
+        <v>-14264.3558075108</v>
       </c>
       <c r="E13" t="n">
-        <v>-12850.779457811</v>
+        <v>-14228.4510757586</v>
       </c>
       <c r="F13" t="n">
-        <v>6449.34209478161</v>
+        <v>7138.17790375541</v>
       </c>
       <c r="G13" t="n">
-        <v>0.00111998708288077</v>
+        <v>0.000501106245189692</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0243912623011049</v>
+        <v>0.0159658731902145</v>
       </c>
       <c r="I13" t="n">
-        <v>2658.54110714379</v>
+        <v>3709.48725401426</v>
       </c>
       <c r="J13" t="n">
         <v>100</v>
@@ -909,31 +891,31 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D14" t="n">
-        <v>-16459.2335450459</v>
+        <v>-21219.4284734558</v>
       </c>
       <c r="E14" t="n">
-        <v>-16423.3288132937</v>
+        <v>-21183.5237417036</v>
       </c>
       <c r="F14" t="n">
-        <v>8235.61677252294</v>
+        <v>10615.7142367279</v>
       </c>
       <c r="G14" t="n">
-        <v>0.000359553633729885</v>
+        <v>0.000022087444096846</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0134005293713835</v>
+        <v>0.00350169636436102</v>
       </c>
       <c r="I14" t="n">
-        <v>3632.91127262384</v>
+        <v>6155.99198275984</v>
       </c>
       <c r="J14" t="n">
         <v>100</v>
@@ -944,31 +926,31 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>-18960.5341690539</v>
+        <v>-21922.1562477529</v>
       </c>
       <c r="E15" t="n">
-        <v>-18924.6294373017</v>
+        <v>-21886.2515160007</v>
       </c>
       <c r="F15" t="n">
-        <v>9486.26708452694</v>
+        <v>10967.0781238764</v>
       </c>
       <c r="G15" t="n">
-        <v>0.000173379545562513</v>
+        <v>0.0000344625055079826</v>
       </c>
       <c r="H15" t="n">
-        <v>0.00874464817762341</v>
+        <v>0.00431020849269093</v>
       </c>
       <c r="I15" t="n">
-        <v>4469.83721075024</v>
+        <v>5798.56273183701</v>
       </c>
       <c r="J15" t="n">
         <v>100</v>
@@ -979,31 +961,31 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
         <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D16" t="n">
-        <v>-15123.4937397722</v>
+        <v>-17933.4795528587</v>
       </c>
       <c r="E16" t="n">
-        <v>-15087.58900802</v>
+        <v>-17897.5748211065</v>
       </c>
       <c r="F16" t="n">
-        <v>7567.7468698861</v>
+        <v>8972.73977642934</v>
       </c>
       <c r="G16" t="n">
-        <v>0.000428298440333085</v>
+        <v>0.0000984774616507493</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0149533648237795</v>
+        <v>0.00763377013464728</v>
       </c>
       <c r="I16" t="n">
-        <v>3705.8767497545</v>
+        <v>4808.33473745732</v>
       </c>
       <c r="J16" t="n">
         <v>100</v>
@@ -1014,7 +996,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
@@ -1023,22 +1005,22 @@
         <v>17</v>
       </c>
       <c r="D17" t="n">
-        <v>-18150.2559713468</v>
+        <v>-13272.5886735945</v>
       </c>
       <c r="E17" t="n">
-        <v>-18114.3512395946</v>
+        <v>-13236.6839418423</v>
       </c>
       <c r="F17" t="n">
-        <v>9081.12798567339</v>
+        <v>6642.29433679725</v>
       </c>
       <c r="G17" t="n">
-        <v>0.000205489863478527</v>
+        <v>0.00111571180507688</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0092717928429477</v>
+        <v>0.0243005150863015</v>
       </c>
       <c r="I17" t="n">
-        <v>4536.71715531798</v>
+        <v>-529.69346230837</v>
       </c>
       <c r="J17" t="n">
         <v>100</v>
@@ -1049,7 +1031,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
         <v>12</v>
@@ -1058,22 +1040,22 @@
         <v>18</v>
       </c>
       <c r="D18" t="n">
-        <v>-14264.3558075108</v>
+        <v>-16714.5673553433</v>
       </c>
       <c r="E18" t="n">
-        <v>-14228.4510757586</v>
+        <v>-16678.6626235911</v>
       </c>
       <c r="F18" t="n">
-        <v>7138.17790375541</v>
+        <v>8363.28367767167</v>
       </c>
       <c r="G18" t="n">
-        <v>0.000499517062406974</v>
+        <v>0.000359467521655461</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0159105849633656</v>
+        <v>0.0133606526697377</v>
       </c>
       <c r="I18" t="n">
-        <v>3667.09004176556</v>
+        <v>3248.81444404427</v>
       </c>
       <c r="J18" t="n">
         <v>100</v>
@@ -1084,31 +1066,31 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D19" t="n">
-        <v>-21922.1562477529</v>
+        <v>-14011.7133296657</v>
       </c>
       <c r="E19" t="n">
-        <v>-21886.2515160007</v>
+        <v>-13975.8085979135</v>
       </c>
       <c r="F19" t="n">
-        <v>10967.0781238764</v>
+        <v>7011.85666483284</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0000345680721357787</v>
+        <v>0.000498570509531138</v>
       </c>
       <c r="H19" t="n">
-        <v>0.00433773410563787</v>
+        <v>0.015920621645987</v>
       </c>
       <c r="I19" t="n">
-        <v>5811.5591325607</v>
+        <v>3634.81880350302</v>
       </c>
       <c r="J19" t="n">
         <v>100</v>
@@ -1119,31 +1101,31 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B20" t="s">
         <v>12</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D20" t="n">
-        <v>-22012.2166080391</v>
+        <v>-21907.805785593</v>
       </c>
       <c r="E20" t="n">
-        <v>-21976.3118762869</v>
+        <v>-21871.9010538407</v>
       </c>
       <c r="F20" t="n">
-        <v>11012.1083040196</v>
+        <v>10959.9028927965</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0000307143365551819</v>
+        <v>0.0000222618338310743</v>
       </c>
       <c r="H20" t="n">
-        <v>0.00410291111855608</v>
+        <v>0.00351574114682221</v>
       </c>
       <c r="I20" t="n">
-        <v>5832.10992128852</v>
+        <v>5757.42286630926</v>
       </c>
       <c r="J20" t="n">
         <v>100</v>
@@ -1154,31 +1136,31 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D21" t="n">
-        <v>-13272.5886735945</v>
+        <v>-22143.852773775</v>
       </c>
       <c r="E21" t="n">
-        <v>-13236.6839418423</v>
+        <v>-22107.9480420228</v>
       </c>
       <c r="F21" t="n">
-        <v>6642.29433679725</v>
+        <v>11077.9263868875</v>
       </c>
       <c r="G21" t="n">
-        <v>0.00111506312641247</v>
+        <v>0.0000342948457725066</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0243114940550477</v>
+        <v>0.00431345636426224</v>
       </c>
       <c r="I21" t="n">
-        <v>-954.938640688398</v>
+        <v>5462.45050322239</v>
       </c>
       <c r="J21" t="n">
         <v>100</v>
@@ -1189,31 +1171,31 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B22" t="s">
         <v>12</v>
       </c>
       <c r="C22" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D22" t="n">
-        <v>-16714.5673553433</v>
+        <v>-18465.0005679739</v>
       </c>
       <c r="E22" t="n">
-        <v>-16678.6626235911</v>
+        <v>-18429.0958362217</v>
       </c>
       <c r="F22" t="n">
-        <v>8363.28367767167</v>
+        <v>9238.50028398695</v>
       </c>
       <c r="G22" t="n">
-        <v>0.000357907528885292</v>
+        <v>0.0000984836619257087</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0133236556785465</v>
+        <v>0.00765067361239577</v>
       </c>
       <c r="I22" t="n">
-        <v>3506.86690699592</v>
+        <v>4609.36250568606</v>
       </c>
       <c r="J22" t="n">
         <v>100</v>
@@ -1224,31 +1206,31 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D23" t="n">
-        <v>-19180.8529014042</v>
+        <v>-13301.5420123857</v>
       </c>
       <c r="E23" t="n">
-        <v>-19144.948169652</v>
+        <v>-13265.6372806335</v>
       </c>
       <c r="F23" t="n">
-        <v>9596.42645070209</v>
+        <v>6656.77100619286</v>
       </c>
       <c r="G23" t="n">
-        <v>0.000173312938629055</v>
+        <v>0.00111858176577476</v>
       </c>
       <c r="H23" t="n">
-        <v>0.00874668437307545</v>
+        <v>0.0243880749955382</v>
       </c>
       <c r="I23" t="n">
-        <v>4067.86518242951</v>
+        <v>1410.21991443546</v>
       </c>
       <c r="J23" t="n">
         <v>100</v>
@@ -1259,31 +1241,31 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>12</v>
       </c>
       <c r="C24" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D24" t="n">
-        <v>-15518.5292120059</v>
+        <v>-16755.7121347858</v>
       </c>
       <c r="E24" t="n">
-        <v>-15482.6244802537</v>
+        <v>-16719.8074030336</v>
       </c>
       <c r="F24" t="n">
-        <v>7765.26460600297</v>
+        <v>8383.85606739289</v>
       </c>
       <c r="G24" t="n">
-        <v>0.000428482527248528</v>
+        <v>0.000358075361711318</v>
       </c>
       <c r="H24" t="n">
-        <v>0.0149318974829823</v>
+        <v>0.013326504407556</v>
       </c>
       <c r="I24" t="n">
-        <v>2857.45024859483</v>
+        <v>2818.3700365612</v>
       </c>
       <c r="J24" t="n">
         <v>100</v>
@@ -1294,456 +1276,36 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
         <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D25" t="n">
-        <v>-18195.3717021399</v>
+        <v>-14556.4722711371</v>
       </c>
       <c r="E25" t="n">
-        <v>-18159.4669703877</v>
+        <v>-14520.5675393849</v>
       </c>
       <c r="F25" t="n">
-        <v>9103.68585106996</v>
+        <v>7284.23613556855</v>
       </c>
       <c r="G25" t="n">
-        <v>0.000205151988665101</v>
+        <v>0.000498260603830628</v>
       </c>
       <c r="H25" t="n">
-        <v>0.00924562488450474</v>
+        <v>0.0158925403058326</v>
       </c>
       <c r="I25" t="n">
-        <v>4510.56549898657</v>
+        <v>3004.53971926223</v>
       </c>
       <c r="J25" t="n">
         <v>100</v>
       </c>
       <c r="K25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" t="s">
-        <v>20</v>
-      </c>
-      <c r="D26" t="n">
-        <v>-21907.805785593</v>
-      </c>
-      <c r="E26" t="n">
-        <v>-21871.9010538407</v>
-      </c>
-      <c r="F26" t="n">
-        <v>10959.9028927965</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0.0000221909262070413</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0.00350857180301007</v>
-      </c>
-      <c r="I26" t="n">
-        <v>5763.22817256436</v>
-      </c>
-      <c r="J26" t="n">
-        <v>100</v>
-      </c>
-      <c r="K26" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" t="s">
-        <v>21</v>
-      </c>
-      <c r="D27" t="n">
-        <v>-22143.852773775</v>
-      </c>
-      <c r="E27" t="n">
-        <v>-22107.9480420228</v>
-      </c>
-      <c r="F27" t="n">
-        <v>11077.9263868875</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0.0000344412906441569</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0.00432088171460377</v>
-      </c>
-      <c r="I27" t="n">
-        <v>5437.85940640172</v>
-      </c>
-      <c r="J27" t="n">
-        <v>100</v>
-      </c>
-      <c r="K27" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s">
-        <v>28</v>
-      </c>
-      <c r="B28" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" t="s">
-        <v>22</v>
-      </c>
-      <c r="D28" t="n">
-        <v>-21895.756317562</v>
-      </c>
-      <c r="E28" t="n">
-        <v>-21859.8515858098</v>
-      </c>
-      <c r="F28" t="n">
-        <v>10953.878158781</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0.0000306445255261147</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0.00409466717270811</v>
-      </c>
-      <c r="I28" t="n">
-        <v>5129.20010934303</v>
-      </c>
-      <c r="J28" t="n">
-        <v>100</v>
-      </c>
-      <c r="K28" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29" t="s">
-        <v>12</v>
-      </c>
-      <c r="C29" t="s">
-        <v>23</v>
-      </c>
-      <c r="D29" t="n">
-        <v>-18465.0005679739</v>
-      </c>
-      <c r="E29" t="n">
-        <v>-18429.0958362217</v>
-      </c>
-      <c r="F29" t="n">
-        <v>9238.50028398695</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0.0000976513819121709</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0.00760844910085838</v>
-      </c>
-      <c r="I29" t="n">
-        <v>4651.52052010725</v>
-      </c>
-      <c r="J29" t="n">
-        <v>100</v>
-      </c>
-      <c r="K29" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="s">
-        <v>28</v>
-      </c>
-      <c r="B30" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" t="s">
-        <v>24</v>
-      </c>
-      <c r="D30" t="n">
-        <v>-18979.930325161</v>
-      </c>
-      <c r="E30" t="n">
-        <v>-18944.0255934088</v>
-      </c>
-      <c r="F30" t="n">
-        <v>9495.96516258049</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0.0000806524470839728</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0.00678442336306669</v>
-      </c>
-      <c r="I30" t="n">
-        <v>4904.74801380754</v>
-      </c>
-      <c r="J30" t="n">
-        <v>100</v>
-      </c>
-      <c r="K30" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="s">
-        <v>28</v>
-      </c>
-      <c r="B31" t="s">
-        <v>12</v>
-      </c>
-      <c r="C31" t="s">
-        <v>25</v>
-      </c>
-      <c r="D31" t="n">
-        <v>-19083.7648599836</v>
-      </c>
-      <c r="E31" t="n">
-        <v>-19047.8601282314</v>
-      </c>
-      <c r="F31" t="n">
-        <v>9547.88242999181</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0.000075701964514223</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0.00658479223177301</v>
-      </c>
-      <c r="I31" t="n">
-        <v>5059.14871156311</v>
-      </c>
-      <c r="J31" t="n">
-        <v>100</v>
-      </c>
-      <c r="K31" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s">
-        <v>28</v>
-      </c>
-      <c r="B32" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" t="n">
-        <v>-13301.5420123857</v>
-      </c>
-      <c r="E32" t="n">
-        <v>-13265.6372806335</v>
-      </c>
-      <c r="F32" t="n">
-        <v>6656.77100619286</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0.00111535198781881</v>
-      </c>
-      <c r="H32" t="n">
-        <v>0.0243461097605127</v>
-      </c>
-      <c r="I32" t="n">
-        <v>1460.89282075391</v>
-      </c>
-      <c r="J32" t="n">
-        <v>100</v>
-      </c>
-      <c r="K32" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s">
-        <v>28</v>
-      </c>
-      <c r="B33" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" t="s">
-        <v>15</v>
-      </c>
-      <c r="D33" t="n">
-        <v>-16755.7121347858</v>
-      </c>
-      <c r="E33" t="n">
-        <v>-16719.8074030336</v>
-      </c>
-      <c r="F33" t="n">
-        <v>8383.85606739289</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0.000358311906816433</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0.0133356319444019</v>
-      </c>
-      <c r="I33" t="n">
-        <v>2738.55288217004</v>
-      </c>
-      <c r="J33" t="n">
-        <v>100</v>
-      </c>
-      <c r="K33" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34" t="s">
-        <v>16</v>
-      </c>
-      <c r="D34" t="n">
-        <v>-19203.1063159103</v>
-      </c>
-      <c r="E34" t="n">
-        <v>-19167.2015841581</v>
-      </c>
-      <c r="F34" t="n">
-        <v>9607.55315795517</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0.000173197985650938</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0.00874048073550589</v>
-      </c>
-      <c r="I34" t="n">
-        <v>3164.23839893327</v>
-      </c>
-      <c r="J34" t="n">
-        <v>100</v>
-      </c>
-      <c r="K34" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s">
-        <v>28</v>
-      </c>
-      <c r="B35" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" t="s">
-        <v>26</v>
-      </c>
-      <c r="D35" t="n">
-        <v>-15580.3567037644</v>
-      </c>
-      <c r="E35" t="n">
-        <v>-15544.4519720122</v>
-      </c>
-      <c r="F35" t="n">
-        <v>7796.17835188222</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0.00042645367996808</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.0148824626149487</v>
-      </c>
-      <c r="I35" t="n">
-        <v>2990.1367093086</v>
-      </c>
-      <c r="J35" t="n">
-        <v>100</v>
-      </c>
-      <c r="K35" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s">
-        <v>28</v>
-      </c>
-      <c r="B36" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" t="n">
-        <v>-18318.3939502536</v>
-      </c>
-      <c r="E36" t="n">
-        <v>-18282.4892185014</v>
-      </c>
-      <c r="F36" t="n">
-        <v>9165.19697512682</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0.000203860081043165</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0.00921797702585573</v>
-      </c>
-      <c r="I36" t="n">
-        <v>3448.12878340455</v>
-      </c>
-      <c r="J36" t="n">
-        <v>100</v>
-      </c>
-      <c r="K36" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="s">
-        <v>28</v>
-      </c>
-      <c r="B37" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" t="s">
-        <v>18</v>
-      </c>
-      <c r="D37" t="n">
-        <v>-14556.4722711371</v>
-      </c>
-      <c r="E37" t="n">
-        <v>-14520.5675393849</v>
-      </c>
-      <c r="F37" t="n">
-        <v>7284.23613556855</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0.000498508651405117</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.0158785332225842</v>
-      </c>
-      <c r="I37" t="n">
-        <v>3007.31078665545</v>
-      </c>
-      <c r="J37" t="n">
-        <v>100</v>
-      </c>
-      <c r="K37" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1766,112 +1328,112 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" t="s">
         <v>29</v>
-      </c>
-      <c r="D1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>-18349.3078348571</v>
+        <v>-17855.0642576084</v>
       </c>
       <c r="D2" t="n">
-        <v>-18313.4031031049</v>
+        <v>-17819.1595258562</v>
       </c>
       <c r="E2" t="n">
-        <v>9180.65391742856</v>
+        <v>8933.53212880421</v>
       </c>
       <c r="F2" t="n">
-        <v>0.000259747235715852</v>
+        <v>0.000354993012140999</v>
       </c>
       <c r="G2" t="n">
-        <v>0.00994191505748577</v>
+        <v>0.0115144984720678</v>
       </c>
       <c r="H2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>-18109.1741651016</v>
+        <v>-17546.387452374</v>
       </c>
       <c r="D3" t="n">
-        <v>-18073.2694333493</v>
+        <v>-17510.4827206217</v>
       </c>
       <c r="E3" t="n">
-        <v>9060.58708255078</v>
+        <v>8779.19372618698</v>
       </c>
       <c r="F3" t="n">
-        <v>0.000260915066165745</v>
+        <v>0.000355772444981603</v>
       </c>
       <c r="G3" t="n">
-        <v>0.00997997001646905</v>
+        <v>0.0115222046259424</v>
       </c>
       <c r="H3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>-18116.6118143257</v>
+        <v>-17512.3222721118</v>
       </c>
       <c r="D4" t="n">
-        <v>-18080.7070825735</v>
+        <v>-17476.4175403596</v>
       </c>
       <c r="E4" t="n">
-        <v>9064.30590716285</v>
+        <v>8762.16113605591</v>
       </c>
       <c r="F4" t="n">
-        <v>0.000335028645504487</v>
+        <v>0.000354796207919843</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0112857145283358</v>
+        <v>0.0115045773989542</v>
       </c>
       <c r="H4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -1882,25 +1444,25 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>-16347.3155700878</v>
+        <v>-17736.2830420607</v>
       </c>
       <c r="D5" t="n">
-        <v>-16317.3949602943</v>
+        <v>-17706.3624322672</v>
       </c>
       <c r="E5" t="n">
-        <v>8178.65778504392</v>
+        <v>8873.14152103034</v>
       </c>
       <c r="F5" t="n">
-        <v>0.00047023782781393</v>
+        <v>0.000354806903204492</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0143034536367556</v>
+        <v>0.0114995209947058</v>
       </c>
       <c r="H5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I5" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>